<commit_message>
Retired status plutôt que suppression pour les artefacts Encounter, changelog
Restaure fr-core-vs-encounter-class, fr-core-vs-encounter-discharge-disposition
et fr-core-cs-circonstances-sortie (déjà publiés en 2.2.0) avec status retired
au lieu de les supprimer, pour éviter de casser leur URL canonique. Les
bindings retirés du profil Encounter ne sont pas réintroduits. Ajoute deux
entrées de changelog : passage en retired de ces artefacts, et assouplissement
de la cardinalité Encounter.period.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> afb93c93fbda197c1ed305fca0b4a58e91d90768
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-22T12:23:37+00:00</t>
+    <t>2026-10-13T09:01:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -949,7 +949,7 @@
     <t>Concepts representing classification of patient encounter such as ambulatory (outpatient), inpatient, emergency, home health or others due to local variations.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActEncounterCode-cisis|20260716085852</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-hl7-v3-ActEncounterCode-cisis|20260916095454</t>
   </si>
   <si>
     <t>.inboundRelationship[typeCode=SUBJ].source[classCode=LIST].code</t>

</xml_diff>